<commit_message>
docs(v1.8.0): freeze employment sites and migration design
</commit_message>
<xml_diff>
--- a/templates/POST-UAT-v1.8.0-UAT-MASTER-DATA-SEED-TEMPLATE.xlsx
+++ b/templates/POST-UAT-v1.8.0-UAT-MASTER-DATA-SEED-TEMPLATE.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rf98d245417304d3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centers" sheetId="2" r:id="Rfeca1f85bc3f4a95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team-Center" sheetId="3" r:id="R44851ef5b81c4b7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Sites" sheetId="4" r:id="Rcda2e1fea80148fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team-Site" sheetId="5" r:id="Rc4868c3cd5e0447b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employment-Primary Site" sheetId="6" r:id="R7c33627d0fa74b28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mileage Rates" sheetId="7" r:id="R48d8d91433604851"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R12b6f179cd1b4747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centers" sheetId="2" r:id="Rc2b097ea2ab1426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team-Center" sheetId="3" r:id="Rfa8beb773818455f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Sites" sheetId="4" r:id="Rc121584855d5447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team-Site" sheetId="5" r:id="R883ec1a9a3c948c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employment-Site" sheetId="6" r:id="Raa823c508d324ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mileage Rates" sheetId="7" r:id="R72bdee7a87434beb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -332,7 +332,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="EmploymentPrimarySiteTable" displayName="EmploymentPrimarySiteTable" ref="A5:F105" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="EmploymentSiteTable" displayName="EmploymentSiteTable" ref="A5:F105" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="OrganizationCode"/>
     <x:tableColumn id="2" name="EmployeeNo"/>
@@ -693,7 +693,7 @@
         <x:v>Effective Team → Site availability</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
-        <x:v>Employment-Primary Site</x:v>
+        <x:v>Employment-Site</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
         <x:v>Not started</x:v>
@@ -704,13 +704,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>Employment-Primary Site</x:v>
+        <x:v>Employment-Site</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
         <x:v>HR/Business</x:v>
       </x:c>
       <x:c r="D10" s="16" t="str">
-        <x:v>Primary Site per Employment</x:v>
+        <x:v>Usable Sites + one Primary per Employment/date</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
         <x:v>UAT import</x:v>
@@ -794,7 +794,7 @@
         <x:v>Periods</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>Dates are inclusive; same-day overlaps are blocked.</x:v>
+        <x:v>Dates are inclusive. Employment-Site allows multiple active assignments, but Primary periods cannot overlap.</x:v>
       </x:c>
       <x:c r="C16" s="16"/>
       <x:c r="D16" s="16"/>
@@ -806,7 +806,7 @@
         <x:v>Keys</x:v>
       </x:c>
       <x:c r="B17" s="16" t="str">
-        <x:v>Codes/EmployeeNo are text. No fuzzy or name-based matching.</x:v>
+        <x:v>Codes/EmployeeNo are text; no fuzzy matching. Every Employment-Site period must be covered by the Employment's effective Team-Site eligibility.</x:v>
       </x:c>
       <x:c r="C17" s="16"/>
       <x:c r="D17" s="16"/>
@@ -1855,7 +1855,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Read7a2c38a564e11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdbedf494ebc444e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2738,7 +2738,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1b6fdeb70024895"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra649164218e24c7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4058,7 +4058,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re16b8a7371774692"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e4c94e49d5a49fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4833,7 +4833,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b68bf81132747f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeed10e5642a47da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4852,7 +4852,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="12" t="str">
-        <x:v>Employment → Primary Deployment Site — HR/Business Input</x:v>
+        <x:v>Employment → Deployment Site — HR/Business Input</x:v>
       </x:c>
       <x:c r="B1" s="13"/>
       <x:c r="C1" s="13"/>
@@ -4862,7 +4862,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="36" t="str">
-        <x:v>Business key: OrganizationCode + EmployeeNo + EffectiveFrom</x:v>
+        <x:v>Business key: OrganizationCode + EmployeeNo + SiteCode + EffectiveFrom</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -4872,7 +4872,7 @@
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
       <x:c r="A3" s="37" t="str">
-        <x:v>One Employment may have only one Primary Site on a date. This sheet does not define secondary assignments.</x:v>
+        <x:v>Multiple active Site assignments are allowed. At most one Primary Site per date; every Site period must be covered by the Employment's effective Team-Site eligibility.</x:v>
       </x:c>
       <x:c r="B3" s="13"/>
       <x:c r="C3" s="13"/>
@@ -5715,13 +5715,13 @@
     <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="D6:D105">
-      <x:formula1>"TRUE"</x:formula1>
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showErrorMessage="1" errorTitle="Invalid IsPrimary value" error="Enter TRUE for the one Primary period or FALSE for another usable Site assignment." sqref="D6:D105">
+      <x:formula1>"TRUE,FALSE"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R613586f04c3643db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dc1304d319e4b84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6720,7 +6720,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0db17427a2f435a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3acba57b93cd46c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>